<commit_message>
included switch between income and tenure classification
</commit_message>
<xml_diff>
--- a/data_input/density_housing_combo_emissions.xlsx
+++ b/data_input/density_housing_combo_emissions.xlsx
@@ -441,22 +441,22 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>highest_income_emission_per_capita</t>
+          <t>highest_classome_emission_per_capita</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>lowest_income_emission_per_capita</t>
+          <t>lowest_classome_emission_per_capita</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>median_income_emission_per_capita</t>
+          <t>median_classome_emission_per_capita</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>mean_income_emission_per_capita</t>
+          <t>mean_classome_emission_per_capita</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
@@ -477,19 +477,19 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>8040.970109387149</v>
+        <v>8198.664246285654</v>
       </c>
       <c r="D2" t="n">
-        <v>5054.282692281504</v>
+        <v>5828.962448591719</v>
       </c>
       <c r="E2" t="n">
-        <v>5885.951898915166</v>
+        <v>6561.570523684385</v>
       </c>
       <c r="F2" t="n">
-        <v>6106.562913768127</v>
+        <v>6863.065739520586</v>
       </c>
       <c r="G2" t="n">
-        <v>349280</v>
+        <v>348795</v>
       </c>
     </row>
     <row r="3">
@@ -504,19 +504,19 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>8121.675126238261</v>
+        <v>7658.941041718369</v>
       </c>
       <c r="D3" t="n">
-        <v>5303.418854321621</v>
+        <v>5450.814615610396</v>
       </c>
       <c r="E3" t="n">
-        <v>6319.162308162297</v>
+        <v>5978.629674116797</v>
       </c>
       <c r="F3" t="n">
-        <v>6318.396236193536</v>
+        <v>6362.795110481854</v>
       </c>
       <c r="G3" t="n">
-        <v>581490</v>
+        <v>580490</v>
       </c>
     </row>
     <row r="4">
@@ -531,19 +531,19 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>8646.154450363323</v>
+        <v>10952.3488207333</v>
       </c>
       <c r="D4" t="n">
-        <v>5928.725363606151</v>
+        <v>6106.514435431332</v>
       </c>
       <c r="E4" t="n">
-        <v>6420.572289941279</v>
+        <v>6377.921629210594</v>
       </c>
       <c r="F4" t="n">
-        <v>6867.551999666795</v>
+        <v>7812.261628458407</v>
       </c>
       <c r="G4" t="n">
-        <v>1289720</v>
+        <v>1287190</v>
       </c>
     </row>
     <row r="5">
@@ -558,19 +558,19 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>7934.693075796217</v>
+        <v>8770.579914911623</v>
       </c>
       <c r="D5" t="n">
-        <v>4826.624927306922</v>
+        <v>5723.081346679503</v>
       </c>
       <c r="E5" t="n">
-        <v>5629.038335365296</v>
+        <v>6696.388540639855</v>
       </c>
       <c r="F5" t="n">
-        <v>5867.712285361025</v>
+        <v>7063.349934076993</v>
       </c>
       <c r="G5" t="n">
-        <v>211740</v>
+        <v>211320</v>
       </c>
     </row>
     <row r="6">
@@ -585,19 +585,19 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>7354.360757457202</v>
+        <v>10987.49189854286</v>
       </c>
       <c r="D6" t="n">
-        <v>4734.777792763417</v>
+        <v>5306.276426189853</v>
       </c>
       <c r="E6" t="n">
-        <v>5206.54277512977</v>
+        <v>7523.491433603667</v>
       </c>
       <c r="F6" t="n">
-        <v>5446.307891052858</v>
+        <v>7939.086586112126</v>
       </c>
       <c r="G6" t="n">
-        <v>35460</v>
+        <v>36340</v>
       </c>
     </row>
     <row r="7">
@@ -612,19 +612,19 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>8018.032507864995</v>
+        <v>7133.277192901137</v>
       </c>
       <c r="D7" t="n">
-        <v>3984.78200720532</v>
+        <v>4716.771949011476</v>
       </c>
       <c r="E7" t="n">
-        <v>5297.036275290679</v>
+        <v>6836.521265689447</v>
       </c>
       <c r="F7" t="n">
-        <v>5607.559789409881</v>
+        <v>6228.85680253402</v>
       </c>
       <c r="G7" t="n">
-        <v>396905</v>
+        <v>395320</v>
       </c>
     </row>
     <row r="8">
@@ -639,19 +639,19 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>8074.544568075141</v>
+        <v>7445.984588877515</v>
       </c>
       <c r="D8" t="n">
-        <v>4615.985435618679</v>
+        <v>5434.811222555813</v>
       </c>
       <c r="E8" t="n">
-        <v>5712.495992447579</v>
+        <v>7149.382960972376</v>
       </c>
       <c r="F8" t="n">
-        <v>6064.649335922133</v>
+        <v>6676.726257468569</v>
       </c>
       <c r="G8" t="n">
-        <v>223770</v>
+        <v>222805</v>
       </c>
     </row>
     <row r="9">
@@ -666,19 +666,19 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>7999.456367683954</v>
+        <v>11944.58732442599</v>
       </c>
       <c r="D9" t="n">
-        <v>5473.771807024237</v>
+        <v>6424.390031906311</v>
       </c>
       <c r="E9" t="n">
-        <v>5849.602621269828</v>
+        <v>6861.832087408879</v>
       </c>
       <c r="F9" t="n">
-        <v>6321.782812496443</v>
+        <v>8410.269814580393</v>
       </c>
       <c r="G9" t="n">
-        <v>136955</v>
+        <v>136165</v>
       </c>
     </row>
     <row r="10">
@@ -693,19 +693,19 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>7736.864472672411</v>
+        <v>6328.114691664112</v>
       </c>
       <c r="D10" t="n">
-        <v>3108.325188511533</v>
+        <v>3830.975120314312</v>
       </c>
       <c r="E10" t="n">
-        <v>4974.670791781698</v>
+        <v>6194.919120435591</v>
       </c>
       <c r="F10" t="n">
-        <v>5128.183981985838</v>
+        <v>5451.336310804672</v>
       </c>
       <c r="G10" t="n">
-        <v>1035935</v>
+        <v>1032780</v>
       </c>
     </row>
     <row r="11">
@@ -720,19 +720,19 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>6170.191555989972</v>
+        <v>5238.971610431654</v>
       </c>
       <c r="D11" t="n">
-        <v>2764.264743548116</v>
+        <v>3293.025163421462</v>
       </c>
       <c r="E11" t="n">
-        <v>3984.047945700943</v>
+        <v>4820.771990037463</v>
       </c>
       <c r="F11" t="n">
-        <v>4194.990009063653</v>
+        <v>4450.922921296859</v>
       </c>
       <c r="G11" t="n">
-        <v>2072825</v>
+        <v>2066805</v>
       </c>
     </row>
     <row r="12">
@@ -747,19 +747,19 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>7003.825419847956</v>
+        <v>4545.758814181378</v>
       </c>
       <c r="D12" t="n">
-        <v>3209.404498934629</v>
+        <v>3310.955528946273</v>
       </c>
       <c r="E12" t="n">
-        <v>4242.569889190398</v>
+        <v>4476.425445977616</v>
       </c>
       <c r="F12" t="n">
-        <v>4657.997796222377</v>
+        <v>4111.046596368422</v>
       </c>
       <c r="G12" t="n">
-        <v>1340025</v>
+        <v>1339450</v>
       </c>
     </row>
     <row r="13">
@@ -774,19 +774,19 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>7155.965375212795</v>
+        <v>4789.753746373264</v>
       </c>
       <c r="D13" t="n">
-        <v>3784.651492219721</v>
+        <v>3542.796449406331</v>
       </c>
       <c r="E13" t="n">
-        <v>4590.098102762888</v>
+        <v>4615.648081507752</v>
       </c>
       <c r="F13" t="n">
-        <v>4987.286686802976</v>
+        <v>4316.066092429116</v>
       </c>
       <c r="G13" t="n">
-        <v>921115</v>
+        <v>920535</v>
       </c>
     </row>
     <row r="14">
@@ -801,19 +801,19 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>7683.052142866337</v>
+        <v>8893.106943405837</v>
       </c>
       <c r="D14" t="n">
-        <v>4503.953234371153</v>
+        <v>4387.595644991877</v>
       </c>
       <c r="E14" t="n">
-        <v>5175.685195999296</v>
+        <v>5280.767692124763</v>
       </c>
       <c r="F14" t="n">
-        <v>5628.950641629022</v>
+        <v>6187.156760174159</v>
       </c>
       <c r="G14" t="n">
-        <v>364975</v>
+        <v>364730</v>
       </c>
     </row>
     <row r="15">
@@ -828,19 +828,19 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>6811.514227246928</v>
+        <v>4455.75129493658</v>
       </c>
       <c r="D15" t="n">
-        <v>2644.48327988148</v>
+        <v>2884.630550941538</v>
       </c>
       <c r="E15" t="n">
-        <v>4053.236552808475</v>
+        <v>4218.698378481555</v>
       </c>
       <c r="F15" t="n">
-        <v>4329.629430158069</v>
+        <v>3853.026741453224</v>
       </c>
       <c r="G15" t="n">
-        <v>1912610</v>
+        <v>1911680</v>
       </c>
     </row>
     <row r="16">
@@ -855,19 +855,19 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>5787.980660137177</v>
+        <v>5757.530811468815</v>
       </c>
       <c r="D16" t="n">
-        <v>2721.527339351564</v>
+        <v>2825.294882776402</v>
       </c>
       <c r="E16" t="n">
-        <v>3620.924995202808</v>
+        <v>3778.160582000226</v>
       </c>
       <c r="F16" t="n">
-        <v>3878.562213503565</v>
+        <v>4120.328758748481</v>
       </c>
       <c r="G16" t="n">
-        <v>954590</v>
+        <v>953795</v>
       </c>
     </row>
     <row r="17">
@@ -882,19 +882,19 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>7320.513607119636</v>
+        <v>5441.569220426625</v>
       </c>
       <c r="D17" t="n">
-        <v>3759.733184154969</v>
+        <v>3788.368017194821</v>
       </c>
       <c r="E17" t="n">
-        <v>4753.474995875225</v>
+        <v>4943.49417043611</v>
       </c>
       <c r="F17" t="n">
-        <v>5121.151373737206</v>
+        <v>4724.477136019185</v>
       </c>
       <c r="G17" t="n">
-        <v>940440</v>
+        <v>939740</v>
       </c>
     </row>
     <row r="18">
@@ -909,19 +909,19 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>7415.75367646327</v>
+        <v>5618.63721107253</v>
       </c>
       <c r="D18" t="n">
-        <v>4362.931397925905</v>
+        <v>4013.159638247409</v>
       </c>
       <c r="E18" t="n">
-        <v>5028.705115725023</v>
+        <v>5133.871531075237</v>
       </c>
       <c r="F18" t="n">
-        <v>5403.289004624383</v>
+        <v>4921.889460131725</v>
       </c>
       <c r="G18" t="n">
-        <v>945900</v>
+        <v>945035</v>
       </c>
     </row>
     <row r="19">
@@ -936,19 +936,19 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>7996.944681002201</v>
+        <v>9490.445059358733</v>
       </c>
       <c r="D19" t="n">
-        <v>5029.898336772986</v>
+        <v>4882.450233503636</v>
       </c>
       <c r="E19" t="n">
-        <v>5576.678897527019</v>
+        <v>5577.023303838034</v>
       </c>
       <c r="F19" t="n">
-        <v>6036.326547942184</v>
+        <v>6649.9728655668</v>
       </c>
       <c r="G19" t="n">
-        <v>760220</v>
+        <v>759325</v>
       </c>
     </row>
     <row r="20">
@@ -963,19 +963,19 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>7160.819969184517</v>
+        <v>5273.848300187878</v>
       </c>
       <c r="D20" t="n">
-        <v>3205.970818840621</v>
+        <v>3340.223653696351</v>
       </c>
       <c r="E20" t="n">
-        <v>4542.632671635328</v>
+        <v>4755.979952271355</v>
       </c>
       <c r="F20" t="n">
-        <v>4804.3770711767</v>
+        <v>4456.683968718527</v>
       </c>
       <c r="G20" t="n">
-        <v>1001340</v>
+        <v>1000540</v>
       </c>
     </row>
     <row r="21">
@@ -990,19 +990,19 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>6303.47580702276</v>
+        <v>6391.93195400605</v>
       </c>
       <c r="D21" t="n">
-        <v>3125.641722341864</v>
+        <v>3206.560618634934</v>
       </c>
       <c r="E21" t="n">
-        <v>4033.422401285551</v>
+        <v>4243.178754697525</v>
       </c>
       <c r="F21" t="n">
-        <v>4318.127119030435</v>
+        <v>4613.89044244617</v>
       </c>
       <c r="G21" t="n">
-        <v>363305</v>
+        <v>363020</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
addded floor area kde to data_explore, added possiblity to merge top1 and deciles
</commit_message>
<xml_diff>
--- a/data_input/density_housing_combo_emissions.xlsx
+++ b/data_input/density_housing_combo_emissions.xlsx
@@ -477,19 +477,19 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>5264.749343899191</v>
+        <v>7022.35421696803</v>
       </c>
       <c r="D2" t="n">
-        <v>3830.670156409551</v>
+        <v>4643.002287088178</v>
       </c>
       <c r="E2" t="n">
-        <v>4164.817632779745</v>
+        <v>4798.163975956058</v>
       </c>
       <c r="F2" t="n">
-        <v>4302.364034194199</v>
+        <v>5487.840160004088</v>
       </c>
       <c r="G2" t="n">
-        <v>368510</v>
+        <v>368380</v>
       </c>
     </row>
     <row r="3">
@@ -504,19 +504,19 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>5711.590216834343</v>
+        <v>6875.952690843332</v>
       </c>
       <c r="D3" t="n">
-        <v>4067.592104677816</v>
+        <v>5175.819918365727</v>
       </c>
       <c r="E3" t="n">
-        <v>4740.400653425189</v>
+        <v>5253.953911800775</v>
       </c>
       <c r="F3" t="n">
-        <v>4804.297503458781</v>
+        <v>5768.575507003278</v>
       </c>
       <c r="G3" t="n">
-        <v>603300</v>
+        <v>603145</v>
       </c>
     </row>
     <row r="4">
@@ -531,19 +531,19 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>6044.486568191954</v>
+        <v>6706.930190072303</v>
       </c>
       <c r="D4" t="n">
-        <v>4355.942734835413</v>
+        <v>5489.877702063777</v>
       </c>
       <c r="E4" t="n">
-        <v>4899.728941589099</v>
+        <v>5902.336447116666</v>
       </c>
       <c r="F4" t="n">
-        <v>4979.302579061574</v>
+        <v>6033.048113084248</v>
       </c>
       <c r="G4" t="n">
-        <v>1308490</v>
+        <v>1307940</v>
       </c>
     </row>
     <row r="5">
@@ -558,19 +558,19 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>5303.059251865821</v>
+        <v>8208.365989629841</v>
       </c>
       <c r="D5" t="n">
-        <v>3894.817204797086</v>
+        <v>4646.171981168795</v>
       </c>
       <c r="E5" t="n">
-        <v>4136.420579707641</v>
+        <v>5929.426064892786</v>
       </c>
       <c r="F5" t="n">
-        <v>4286.521579007051</v>
+        <v>6261.321345230474</v>
       </c>
       <c r="G5" t="n">
-        <v>224425</v>
+        <v>224295</v>
       </c>
     </row>
     <row r="6">
@@ -585,19 +585,19 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>4896.879161977036</v>
+        <v>9377.689862340778</v>
       </c>
       <c r="D6" t="n">
-        <v>3460.790363030416</v>
+        <v>4428.303923288431</v>
       </c>
       <c r="E6" t="n">
-        <v>3777.295002653244</v>
+        <v>6263.467842375323</v>
       </c>
       <c r="F6" t="n">
-        <v>3883.458337292327</v>
+        <v>6689.820542668177</v>
       </c>
       <c r="G6" t="n">
-        <v>43755</v>
+        <v>44345</v>
       </c>
     </row>
     <row r="7">
@@ -612,19 +612,19 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>6397.304732007802</v>
+        <v>5885.438713979452</v>
       </c>
       <c r="D7" t="n">
-        <v>3266.873600760683</v>
+        <v>4039.675989229487</v>
       </c>
       <c r="E7" t="n">
-        <v>4845.355382615042</v>
+        <v>5540.660374485881</v>
       </c>
       <c r="F7" t="n">
-        <v>4721.562472447142</v>
+        <v>5155.258359231607</v>
       </c>
       <c r="G7" t="n">
-        <v>403500</v>
+        <v>402930</v>
       </c>
     </row>
     <row r="8">
@@ -639,19 +639,19 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>7471.834488895447</v>
+        <v>6856.560316007463</v>
       </c>
       <c r="D8" t="n">
-        <v>4082.480497474141</v>
+        <v>5490.845356833731</v>
       </c>
       <c r="E8" t="n">
-        <v>5538.813577526311</v>
+        <v>6472.94577069446</v>
       </c>
       <c r="F8" t="n">
-        <v>5614.436155016505</v>
+        <v>6273.450481178552</v>
       </c>
       <c r="G8" t="n">
-        <v>222185</v>
+        <v>221950</v>
       </c>
     </row>
     <row r="9">
@@ -666,19 +666,19 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>6450.748969703031</v>
+        <v>6544.393529997739</v>
       </c>
       <c r="D9" t="n">
-        <v>4418.243659221745</v>
+        <v>5811.008847314267</v>
       </c>
       <c r="E9" t="n">
-        <v>5020.981111901533</v>
+        <v>5991.233202686336</v>
       </c>
       <c r="F9" t="n">
-        <v>5156.509926965167</v>
+        <v>6115.545193332781</v>
       </c>
       <c r="G9" t="n">
-        <v>145970</v>
+        <v>145890</v>
       </c>
     </row>
     <row r="10">
@@ -693,19 +693,19 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>6247.778002951329</v>
+        <v>5735.381717538879</v>
       </c>
       <c r="D10" t="n">
-        <v>2949.710097990751</v>
+        <v>3567.380433289679</v>
       </c>
       <c r="E10" t="n">
-        <v>4333.568451733792</v>
+        <v>5585.02341419302</v>
       </c>
       <c r="F10" t="n">
-        <v>4407.045840474364</v>
+        <v>4962.595188340526</v>
       </c>
       <c r="G10" t="n">
-        <v>1022305</v>
+        <v>1021385</v>
       </c>
     </row>
     <row r="11">
@@ -720,19 +720,19 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>4707.823492620956</v>
+        <v>4468.895865610992</v>
       </c>
       <c r="D11" t="n">
-        <v>2340.045845033093</v>
+        <v>3000.201665914263</v>
       </c>
       <c r="E11" t="n">
-        <v>3373.583239572061</v>
+        <v>4237.505181626087</v>
       </c>
       <c r="F11" t="n">
-        <v>3377.494167872124</v>
+        <v>3902.200904383781</v>
       </c>
       <c r="G11" t="n">
-        <v>2263780</v>
+        <v>2260775</v>
       </c>
     </row>
     <row r="12">
@@ -747,19 +747,19 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>4661.161182050686</v>
+        <v>3815.326299624254</v>
       </c>
       <c r="D12" t="n">
-        <v>2334.51534600951</v>
+        <v>2755.057301259241</v>
       </c>
       <c r="E12" t="n">
-        <v>3262.190323686394</v>
+        <v>3630.09418701205</v>
       </c>
       <c r="F12" t="n">
-        <v>3343.784769159477</v>
+        <v>3400.159262631848</v>
       </c>
       <c r="G12" t="n">
-        <v>1332375</v>
+        <v>1332050</v>
       </c>
     </row>
     <row r="13">
@@ -774,19 +774,19 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>5338.86523336984</v>
+        <v>4517.508062458724</v>
       </c>
       <c r="D13" t="n">
-        <v>2745.113879639363</v>
+        <v>3441.688371424738</v>
       </c>
       <c r="E13" t="n">
-        <v>3688.18016525343</v>
+        <v>3891.541550423678</v>
       </c>
       <c r="F13" t="n">
-        <v>3961.460962142693</v>
+        <v>3950.245994769046</v>
       </c>
       <c r="G13" t="n">
-        <v>883200</v>
+        <v>883000</v>
       </c>
     </row>
     <row r="14">
@@ -801,19 +801,19 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>5841.020028160136</v>
+        <v>4854.986454913957</v>
       </c>
       <c r="D14" t="n">
-        <v>3460.734326983153</v>
+        <v>3860.128216891741</v>
       </c>
       <c r="E14" t="n">
-        <v>4242.076450631436</v>
+        <v>4579.438194532134</v>
       </c>
       <c r="F14" t="n">
-        <v>4318.44146345422</v>
+        <v>4431.51762211261</v>
       </c>
       <c r="G14" t="n">
-        <v>354285</v>
+        <v>354125</v>
       </c>
     </row>
     <row r="15">
@@ -828,19 +828,19 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>4531.038702487694</v>
+        <v>4116.620398576352</v>
       </c>
       <c r="D15" t="n">
-        <v>2256.984794817912</v>
+        <v>2555.855974029972</v>
       </c>
       <c r="E15" t="n">
-        <v>2958.317564648863</v>
+        <v>3642.814579523156</v>
       </c>
       <c r="F15" t="n">
-        <v>3166.778402062278</v>
+        <v>3438.430317376493</v>
       </c>
       <c r="G15" t="n">
-        <v>1908625</v>
+        <v>1908060</v>
       </c>
     </row>
     <row r="16">
@@ -855,19 +855,19 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>3860.202402977864</v>
+        <v>4441.78772480292</v>
       </c>
       <c r="D16" t="n">
-        <v>2101.120858799821</v>
+        <v>2396.895055655953</v>
       </c>
       <c r="E16" t="n">
-        <v>2693.41891369356</v>
+        <v>3334.619606783634</v>
       </c>
       <c r="F16" t="n">
-        <v>2753.638290853633</v>
+        <v>3391.100795747503</v>
       </c>
       <c r="G16" t="n">
-        <v>1062765</v>
+        <v>1062415</v>
       </c>
     </row>
     <row r="17">
@@ -882,19 +882,19 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>4846.402205017375</v>
+        <v>4350.128307305845</v>
       </c>
       <c r="D17" t="n">
-        <v>2763.618906322488</v>
+        <v>3135.222149768143</v>
       </c>
       <c r="E17" t="n">
-        <v>3557.34926193782</v>
+        <v>4070.979075459233</v>
       </c>
       <c r="F17" t="n">
-        <v>3641.825621019407</v>
+        <v>3852.109844177741</v>
       </c>
       <c r="G17" t="n">
-        <v>964030</v>
+        <v>963910</v>
       </c>
     </row>
     <row r="18">
@@ -909,19 +909,19 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>5330.366694522197</v>
+        <v>4794.614216689673</v>
       </c>
       <c r="D18" t="n">
-        <v>3223.338522466793</v>
+        <v>3828.827483170746</v>
       </c>
       <c r="E18" t="n">
-        <v>4018.190641115771</v>
+        <v>4705.927771897054</v>
       </c>
       <c r="F18" t="n">
-        <v>4204.709988150263</v>
+        <v>4443.123157252491</v>
       </c>
       <c r="G18" t="n">
-        <v>947525</v>
+        <v>947310</v>
       </c>
     </row>
     <row r="19">
@@ -936,19 +936,19 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>5803.112968791757</v>
+        <v>5448.115574969082</v>
       </c>
       <c r="D19" t="n">
-        <v>3907.66985185382</v>
+        <v>4254.760218060303</v>
       </c>
       <c r="E19" t="n">
-        <v>4393.594008573393</v>
+        <v>4977.488790525601</v>
       </c>
       <c r="F19" t="n">
-        <v>4500.868224828218</v>
+        <v>4893.454861184995</v>
       </c>
       <c r="G19" t="n">
-        <v>753085</v>
+        <v>752835</v>
       </c>
     </row>
     <row r="20">
@@ -963,19 +963,19 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>4848.937961188008</v>
+        <v>4790.805213748644</v>
       </c>
       <c r="D20" t="n">
-        <v>2677.409512215666</v>
+        <v>2920.039051266024</v>
       </c>
       <c r="E20" t="n">
-        <v>3340.064215164357</v>
+        <v>4006.357503328596</v>
       </c>
       <c r="F20" t="n">
-        <v>3527.72013499107</v>
+        <v>3905.733922781088</v>
       </c>
       <c r="G20" t="n">
-        <v>1023385</v>
+        <v>1023225</v>
       </c>
     </row>
     <row r="21">
@@ -990,19 +990,19 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>4220.49870381027</v>
+        <v>4956.602588968701</v>
       </c>
       <c r="D21" t="n">
-        <v>2424.545453717012</v>
+        <v>2719.682303042932</v>
       </c>
       <c r="E21" t="n">
-        <v>3026.661757623091</v>
+        <v>3675.464159007716</v>
       </c>
       <c r="F21" t="n">
-        <v>3085.263351394929</v>
+        <v>3783.916350339783</v>
       </c>
       <c r="G21" t="n">
-        <v>411935</v>
+        <v>411890</v>
       </c>
     </row>
   </sheetData>

</xml_diff>